<commit_message>
feat: manual cost editing throughout dashboard
- PUT /api/orders/:id/cost: dedicated cost update endpoint
- OrderDetailPage: '💰 Delivery Cost' section with current value + edit input
- OrdersPage assign modal: 'Delivery cost' field — set cost when assigning rider
- Bulk import: now parses cost_ghs column from template
- Excel template: added cost_ghs column with examples

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/apps/frontend/public/PullUp_Bulk_Order_Template.xlsx
+++ b/apps/frontend/public/PullUp_Bulk_Order_Template.xlsx
@@ -398,9 +398,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -431,134 +431,147 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Save the file and upload it in the admin dashboard under Orders &gt; Import CSV</v>
+        <v>3. Save as CSV (File → Save As → CSV UTF-8) then upload in Settings → Bulk order import</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>4. Sender phone and recipient phone must include country code e.g. +233201234567</v>
+        <v>4. Phone numbers must include country code e.g. +233201234567</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5. Payment method: use cod (cash on delivery) or prepaid</v>
+        <v>5. payment_method: cod (Cash on Delivery) or prepaid</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6. Weight in kg (optional) — add for heavy items over 5kg (surcharge applies)</v>
+        <v>6. cost_ghs: delivery fee in Ghana Cedis (optional — can be set later)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>7. weight_kg: in kilograms (optional, surcharge applies over 5kg)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>COLUMN GUIDE:</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sender_name *</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Full name of the person sending the package</v>
+        <v>COLUMN GUIDE:</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>sender_phone *</v>
+        <v>sender_name *</v>
       </c>
       <c r="B13" t="str">
-        <v>Phone number of the sender e.g. +233201234567</v>
+        <v>Full name of the person sending</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sender_address *</v>
+        <v>sender_phone *</v>
       </c>
       <c r="B14" t="str">
-        <v>Pickup address / location</v>
+        <v>Phone number of sender e.g. +233201234567</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>recipient_name *</v>
+        <v>sender_address *</v>
       </c>
       <c r="B15" t="str">
-        <v>Full name of the person receiving the package</v>
+        <v>Pickup address / location</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>recipient_phone *</v>
+        <v>recipient_name *</v>
       </c>
       <c r="B16" t="str">
-        <v>Phone number of the recipient e.g. +233244987654</v>
+        <v>Full name of the recipient</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>recipient_address *</v>
+        <v>recipient_phone *</v>
       </c>
       <c r="B17" t="str">
-        <v>Delivery address / location</v>
+        <v>Phone number of recipient</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>description *</v>
+        <v>recipient_address *</v>
       </c>
       <c r="B18" t="str">
-        <v>What is being delivered e.g. Documents, Electronics, Food</v>
+        <v>Delivery address</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>weight_kg</v>
+        <v>description *</v>
       </c>
       <c r="B19" t="str">
-        <v>Weight in kilograms (optional, default 0)</v>
+        <v>What is being delivered</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>payment_method *</v>
+        <v>weight_kg</v>
       </c>
       <c r="B20" t="str">
-        <v>cod = Cash on Delivery | prepaid = Already paid</v>
+        <v>Weight in kg (optional)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>special_instructions</v>
+        <v>cost_ghs</v>
       </c>
       <c r="B21" t="str">
-        <v>Any notes for the rider (optional)</v>
+        <v>Delivery fee in GHS (optional, e.g. 45.00)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>payment_method *</v>
+      </c>
+      <c r="B22" t="str">
+        <v>cod = Cash on Delivery | prepaid = Already paid</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Need help? Contact: support@aegisassetllc.com</v>
+        <v>special_instructions</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Notes for rider (optional)</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Questions? Contact: support@aegisassetllc.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -568,8 +581,9 @@
     <col min="6" max="6" width="35.83203125" customWidth="1"/>
     <col min="7" max="7" width="25.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -598,9 +612,12 @@
         <v>weight_kg</v>
       </c>
       <c r="I1" t="str">
+        <v>cost_ghs</v>
+      </c>
+      <c r="J1" t="str">
         <v>payment_method *</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>special_instructions</v>
       </c>
     </row>
@@ -630,9 +647,12 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v>45.00</v>
+      </c>
+      <c r="J2" t="str">
         <v>cod</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v/>
       </c>
     </row>
@@ -662,9 +682,12 @@
         <v>1.5</v>
       </c>
       <c r="I3" t="str">
+        <v>60.00</v>
+      </c>
+      <c r="J3" t="str">
         <v>prepaid</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Call before arrival</v>
       </c>
     </row>
@@ -699,6 +722,9 @@
       <c r="J4" t="str">
         <v/>
       </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -731,6 +757,9 @@
       <c r="J5" t="str">
         <v/>
       </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -763,6 +792,9 @@
       <c r="J6" t="str">
         <v/>
       </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -795,6 +827,9 @@
       <c r="J7" t="str">
         <v/>
       </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -827,6 +862,9 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -859,6 +897,9 @@
       <c r="J9" t="str">
         <v/>
       </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -891,6 +932,9 @@
       <c r="J10" t="str">
         <v/>
       </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -923,10 +967,13 @@
       <c r="J11" t="str">
         <v/>
       </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>